<commit_message>
Implemented XIRR calculation using PYXIRR
</commit_message>
<xml_diff>
--- a/sharesExplorer/sampleFiles/SharePurchasesSampleFile.xlsx
+++ b/sharesExplorer/sampleFiles/SharePurchasesSampleFile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kanaganayagamjanakan/Documents/SoftwareEngineering/Source Codes/SharesExplorer/sharesExplorer/sampleFiles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u79396\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08B32526-7411-DD48-8C90-77E8452E9A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{259A45A8-622F-4207-AB4C-1BA01A483176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17600" activeTab="2" xr2:uid="{1B98F30A-CD37-7F4B-9753-B078AFBAA1D5}"/>
+    <workbookView xWindow="5655" yWindow="3705" windowWidth="21600" windowHeight="11325" activeTab="1" xr2:uid="{1B98F30A-CD37-7F4B-9753-B078AFBAA1D5}"/>
   </bookViews>
   <sheets>
     <sheet name="purchases" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="15">
   <si>
     <t>units</t>
   </si>
@@ -73,12 +73,6 @@
   </si>
   <si>
     <t>29M</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Total</t>
   </si>
   <si>
     <t>price</t>
@@ -100,7 +94,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -504,25 +498,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCCBA220-272A-8947-9BBC-33EF03D4881E}">
   <dimension ref="A1:G76"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="2" max="2" width="28.6640625" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" style="3"/>
+    <col min="2" max="2" width="28.625" customWidth="1"/>
+    <col min="4" max="4" width="18.625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="8" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="8" customFormat="1" ht="18.75">
       <c r="A1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>3</v>
@@ -531,7 +525,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="1">
         <v>44448</v>
       </c>
@@ -552,7 +546,7 @@
         <v>942.4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="1">
         <v>44461</v>
       </c>
@@ -573,7 +567,7 @@
         <v>330.5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="1">
         <v>44470</v>
       </c>
@@ -594,7 +588,7 @@
         <v>522.64</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="1">
         <v>44494</v>
       </c>
@@ -615,7 +609,7 @@
         <v>701.2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="1">
         <v>44519</v>
       </c>
@@ -636,7 +630,7 @@
         <v>599.5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="1">
         <v>44553</v>
       </c>
@@ -657,306 +651,306 @@
         <v>1346.43</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="1"/>
       <c r="D8" s="2"/>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="1"/>
       <c r="D9" s="2"/>
       <c r="F9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="1"/>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="1"/>
       <c r="D11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" s="1"/>
       <c r="D12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" s="1"/>
       <c r="D13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" s="1"/>
       <c r="D14" s="2"/>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" s="1"/>
       <c r="D15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" s="1"/>
       <c r="D16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7">
       <c r="A17" s="1"/>
       <c r="D17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7">
       <c r="A18" s="1"/>
       <c r="D18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7">
       <c r="A19" s="1"/>
       <c r="D19" s="5"/>
       <c r="F19" s="5"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7">
       <c r="A20" s="1"/>
       <c r="D20" s="5"/>
       <c r="F20" s="5"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7">
       <c r="A21" s="1"/>
       <c r="D21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7">
       <c r="A22" s="1"/>
       <c r="D22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7">
       <c r="A23" s="1"/>
       <c r="D23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7">
       <c r="A24" s="1"/>
       <c r="D24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7">
       <c r="A25" s="1"/>
       <c r="D25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7">
       <c r="A27" s="1"/>
       <c r="F27" s="5"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7">
       <c r="A28" s="1"/>
       <c r="D28" s="5"/>
       <c r="F28" s="5"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7">
       <c r="A29" s="1"/>
       <c r="F29" s="5"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7">
       <c r="A30" s="1"/>
       <c r="F30" s="5"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7">
       <c r="A31" s="1"/>
       <c r="F31" s="5"/>
       <c r="G31" s="7"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7">
       <c r="A32" s="1"/>
       <c r="B32" s="5"/>
       <c r="F32" s="5"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6">
       <c r="A33" s="1"/>
       <c r="F33" s="5"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6">
       <c r="A34" s="1"/>
       <c r="F34" s="5"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6">
       <c r="A35" s="1"/>
       <c r="F35" s="5"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6">
       <c r="A36" s="1"/>
       <c r="F36" s="5"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6">
       <c r="A37" s="1"/>
       <c r="F37" s="5"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6">
       <c r="A38" s="1"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6">
       <c r="A39" s="1"/>
       <c r="D39" s="2"/>
       <c r="F39" s="5"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6">
       <c r="A40" s="1"/>
       <c r="D40" s="5"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6">
       <c r="A42" s="1"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6">
       <c r="A43" s="1"/>
       <c r="F43" s="5"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6">
       <c r="A44" s="1"/>
       <c r="F44" s="5"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6">
       <c r="A45" s="1"/>
       <c r="F45" s="5"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6">
       <c r="A46" s="1"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6">
       <c r="A47" s="1"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6">
       <c r="A48" s="1"/>
       <c r="D48" s="5"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6">
       <c r="A49" s="1"/>
       <c r="B49" s="5"/>
       <c r="D49" s="5"/>
       <c r="F49" s="5"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6">
       <c r="A50" s="1"/>
       <c r="D50" s="5"/>
       <c r="F50" s="5"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6">
       <c r="A51" s="1"/>
       <c r="D51" s="5"/>
       <c r="F51" s="5"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6">
       <c r="A52" s="1"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6">
       <c r="A53" s="1"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6">
       <c r="A54" s="1"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6">
       <c r="A55" s="1"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6">
       <c r="A56" s="1"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6">
       <c r="A57" s="1"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6">
       <c r="A58" s="1"/>
       <c r="D58" s="5"/>
       <c r="F58" s="5"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6">
       <c r="A59" s="1"/>
       <c r="F59" s="5"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6">
       <c r="A60" s="1"/>
       <c r="D60" s="5"/>
       <c r="F60" s="5"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6">
       <c r="A61" s="1"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6">
       <c r="A62" s="1"/>
       <c r="D62" s="5"/>
       <c r="F62" s="10"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6">
       <c r="A63" s="1"/>
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
       <c r="F63" s="5"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6">
       <c r="A64" s="1"/>
       <c r="F64" s="10"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6">
       <c r="A65" s="1"/>
       <c r="F65" s="5"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6">
       <c r="A66" s="1"/>
       <c r="D66" s="5"/>
       <c r="F66" s="10"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6">
       <c r="A67" s="1"/>
       <c r="D67" s="5"/>
       <c r="F67" s="5"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6">
       <c r="A68" s="1"/>
       <c r="D68" s="5"/>
       <c r="F68" s="5"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6">
       <c r="A69" s="1"/>
       <c r="D69" s="5"/>
       <c r="F69" s="5"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6">
       <c r="A70" s="1"/>
       <c r="D70" s="5"/>
       <c r="F70" s="5"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6">
       <c r="A71" s="1"/>
       <c r="D71" s="11"/>
       <c r="F71" s="11"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6">
       <c r="A72" s="1"/>
       <c r="D72" s="11"/>
       <c r="F72" s="12"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6">
       <c r="A73" s="1"/>
       <c r="D73" s="11"/>
       <c r="F73" s="11"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6">
       <c r="A74" s="1"/>
       <c r="D74" s="11"/>
       <c r="F74" s="12"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6">
       <c r="A75" s="1"/>
       <c r="D75" s="11"/>
       <c r="F75" s="11"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6">
       <c r="A76" s="1"/>
     </row>
   </sheetData>
@@ -967,24 +961,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF60A9AA-46D5-914E-9B4B-2288670016D3}">
   <dimension ref="A1:C72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="9" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" s="9" customFormat="1">
       <c r="A1" s="9" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" s="1">
         <v>44487</v>
       </c>
@@ -995,7 +989,7 @@
         <v>30.13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3">
       <c r="A3" s="1">
         <v>44580</v>
       </c>
@@ -1006,7 +1000,7 @@
         <v>9.16</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3">
       <c r="A4" s="1">
         <v>44589</v>
       </c>
@@ -1017,207 +1011,207 @@
         <v>3.32</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3">
       <c r="A13" s="1"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3">
       <c r="A14" s="1"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3">
       <c r="A15" s="1"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3">
       <c r="A16" s="1"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1">
       <c r="A17" s="1"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1">
       <c r="A18" s="1"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1">
       <c r="A19" s="1"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1">
       <c r="A20" s="1"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1">
       <c r="A21" s="1"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1">
       <c r="A22" s="1"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1">
       <c r="A23" s="1"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1">
       <c r="A24" s="1"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:1">
       <c r="A25" s="1"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:1">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:1">
       <c r="A28" s="1"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:1">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:1">
       <c r="A30" s="1"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:1">
       <c r="A31" s="1"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:1">
       <c r="A32" s="1"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:1">
       <c r="A33" s="1"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:1">
       <c r="A34" s="1"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:1">
       <c r="A35" s="1"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:1">
       <c r="A36" s="1"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:1">
       <c r="A37" s="1"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:1">
       <c r="A38" s="1"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:1">
       <c r="A39" s="1"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:1">
       <c r="A40" s="1"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:1">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:1">
       <c r="A42" s="1"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:1">
       <c r="A43" s="1"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:1">
       <c r="A44" s="1"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:1">
       <c r="A45" s="1"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:1">
       <c r="A46" s="1"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:1">
       <c r="A47" s="1"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:1">
       <c r="A48" s="1"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:1">
       <c r="A49" s="1"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:1">
       <c r="A50" s="1"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:1">
       <c r="A51" s="1"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:1">
       <c r="A52" s="1"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:1">
       <c r="A53" s="1"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:1">
       <c r="A54" s="1"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:1">
       <c r="A55" s="1"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:1">
       <c r="A56" s="1"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:1">
       <c r="A57" s="1"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:1">
       <c r="A58" s="1"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:1">
       <c r="A59" s="1"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:1">
       <c r="A60" s="1"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:1">
       <c r="A61" s="1"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:1">
       <c r="A62" s="1"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:1">
       <c r="A63" s="1"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:1">
       <c r="A64" s="1"/>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3">
       <c r="A65" s="1"/>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3">
       <c r="A66" s="1"/>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3">
       <c r="A67" s="1"/>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3">
       <c r="A68" s="1"/>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:3">
       <c r="A69" s="1"/>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3">
       <c r="A70" s="1"/>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>11</v>
+    <row r="72" spans="1:3">
+      <c r="B72" t="s">
+        <v>4</v>
       </c>
       <c r="C72">
         <f>SUM(C2:C71)</f>
@@ -1233,25 +1227,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11CD24FB-43DC-1545-8C37-CCACE2AC1261}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="2" max="2" width="28.6640625" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" style="3"/>
+    <col min="2" max="2" width="28.625" customWidth="1"/>
+    <col min="4" max="4" width="18.625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="6" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="6" customFormat="1" ht="18.75">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>3</v>
@@ -1260,12 +1254,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="1">
         <v>45296</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>24</v>
@@ -1281,12 +1275,12 @@
         <v>691.73</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="1">
         <v>45302</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C3">
         <v>1300</v>
@@ -1302,7 +1296,7 @@
         <v>879.01</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="1">
         <v>45315</v>
       </c>
@@ -1323,58 +1317,58 @@
         <v>250.01</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="1"/>
       <c r="D5" s="5"/>
       <c r="F5" s="10"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="1"/>
       <c r="D6" s="2"/>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="1"/>
       <c r="D7" s="2"/>
       <c r="F7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="1"/>
       <c r="D8" s="2"/>
       <c r="F8" s="10"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="1"/>
       <c r="D9" s="2"/>
       <c r="F9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="1"/>
       <c r="D10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="1"/>
       <c r="D11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" s="1"/>
       <c r="F12" s="5"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" s="1"/>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" s="1"/>
       <c r="F14" s="5"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" s="1"/>
       <c r="F15" s="5"/>
     </row>
-    <row r="17" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="5:6">
       <c r="E17">
         <f>SUM(E2:E11)</f>
         <v>14.970000000000141</v>

</xml_diff>